<commit_message>
🔄 Atualização automática - 08/06/2026 08:40:56 (Horário de Brasília)
</commit_message>
<xml_diff>
--- a/dados/indicadores_sao_leopoldo.xlsx
+++ b/dados/indicadores_sao_leopoldo.xlsx
@@ -473,19 +473,19 @@
         <v>2023</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>571</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>417</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
🔄 Atualização automática - 08/06/2026 09:14:47 (Horário de Brasília)
</commit_message>
<xml_diff>
--- a/dados/indicadores_sao_leopoldo.xlsx
+++ b/dados/indicadores_sao_leopoldo.xlsx
@@ -473,19 +473,19 @@
         <v>2023</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>571</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4">

</xml_diff>

<commit_message>
🔄 Atualização automática - 12/06/2026 07:15:56 (Horário de Brasília)
</commit_message>
<xml_diff>
--- a/dados/indicadores_sao_leopoldo.xlsx
+++ b/dados/indicadores_sao_leopoldo.xlsx
@@ -519,13 +519,13 @@
         <v>8</v>
       </c>
       <c r="D5" t="n">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="E5" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F5" t="n">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="6">
@@ -536,16 +536,16 @@
         <v>0</v>
       </c>
       <c r="C6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>205</v>
+        <v>251</v>
       </c>
       <c r="E6" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F6" t="n">
-        <v>106</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🔄 Atualização automática - 09/07/2026 23:39:32 (Horário de Brasília)
</commit_message>
<xml_diff>
--- a/dados/indicadores_sao_leopoldo.xlsx
+++ b/dados/indicadores_sao_leopoldo.xlsx
@@ -519,7 +519,7 @@
         <v>8</v>
       </c>
       <c r="D5" t="n">
-        <v>649</v>
+        <v>651</v>
       </c>
       <c r="E5" t="n">
         <v>54</v>
@@ -539,13 +539,13 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>251</v>
+        <v>296</v>
       </c>
       <c r="E6" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="F6" t="n">
-        <v>121</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
🔄 Atualização automática - 13/08/2026 22:39:09 (Horário de Brasília)
</commit_message>
<xml_diff>
--- a/dados/indicadores_sao_leopoldo.xlsx
+++ b/dados/indicadores_sao_leopoldo.xlsx
@@ -539,13 +539,13 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>296</v>
+        <v>338</v>
       </c>
       <c r="E6" t="n">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="F6" t="n">
-        <v>148</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>

</xml_diff>